<commit_message>
backup step before pruning
</commit_message>
<xml_diff>
--- a/tables/Table 1 Regional cerebral metabolic rates corresponding volume terms and data sources.xlsx
+++ b/tables/Table 1 Regional cerebral metabolic rates corresponding volume terms and data sources.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t xml:space="preserve">Table 1. Regional cerebral metabolic rates, corresponding volume terms and data sources.</t>
   </si>
@@ -32,6 +32,15 @@
     <t xml:space="preserve">mean (both hemispheres)</t>
   </si>
   <si>
+    <t xml:space="preserve">Cerebellum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nucleus dentatus cerebelli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matano et al. 1985 a</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cerebral cortex (global average)</t>
   </si>
   <si>
@@ -146,16 +155,10 @@
     <t xml:space="preserve">Cerebellum1</t>
   </si>
   <si>
-    <t xml:space="preserve">Cerebellum</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cerebellar cortex</t>
   </si>
   <si>
     <t xml:space="preserve">Vermis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nucleus dentatus cerebelli</t>
   </si>
   <si>
     <t xml:space="preserve">White matter</t>
@@ -566,9 +569,11 @@
         <v>6</v>
       </c>
       <c r="B5"/>
-      <c r="C5"/>
+      <c r="C5" t="s">
+        <v>7</v>
+      </c>
       <c r="D5" s="2" t="n">
-        <v>33.5</v>
+        <v>24.2</v>
       </c>
       <c r="E5" t="s">
         <v>7</v>
@@ -578,25 +583,29 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6"/>
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
       <c r="B6"/>
-      <c r="C6" t="s">
-        <v>9</v>
-      </c>
+      <c r="C6"/>
       <c r="D6" s="2" t="n">
-        <v>35.3</v>
-      </c>
-      <c r="E6"/>
-      <c r="F6"/>
+        <v>33.5</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7"/>
       <c r="B7"/>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>35.8</v>
+        <v>35.3</v>
       </c>
       <c r="E7"/>
       <c r="F7"/>
@@ -605,10 +614,10 @@
       <c r="A8"/>
       <c r="B8"/>
       <c r="C8" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>30.5</v>
+        <v>35.8</v>
       </c>
       <c r="E8"/>
       <c r="F8"/>
@@ -617,17 +626,13 @@
       <c r="A9"/>
       <c r="B9"/>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="E9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" t="s">
-        <v>14</v>
-      </c>
+        <v>30.5</v>
+      </c>
+      <c r="E9"/>
+      <c r="F9"/>
     </row>
     <row r="10">
       <c r="A10"/>
@@ -636,7 +641,7 @@
         <v>15</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>30.3</v>
+        <v>35.8</v>
       </c>
       <c r="E10" t="s">
         <v>16</v>
@@ -652,61 +657,65 @@
         <v>18</v>
       </c>
       <c r="D11" s="2" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="E11" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12"/>
+      <c r="B12"/>
+      <c r="C12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="2" t="n">
         <v>25.7</v>
       </c>
-      <c r="E11" t="s">
-        <v>18</v>
-      </c>
-      <c r="F11" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12"/>
-      <c r="C12"/>
-      <c r="D12" s="2"/>
-      <c r="E12"/>
-      <c r="F12"/>
+      <c r="E12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13"/>
-      <c r="B13" t="s">
-        <v>21</v>
-      </c>
+      <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13"/>
       <c r="C13"/>
-      <c r="D13" s="2" t="n">
-        <v>36.2663366336634</v>
-      </c>
-      <c r="E13" t="s">
-        <v>22</v>
-      </c>
-      <c r="F13" t="s">
-        <v>19</v>
-      </c>
+      <c r="D13" s="2"/>
+      <c r="E13"/>
+      <c r="F13"/>
     </row>
     <row r="14">
       <c r="A14"/>
-      <c r="B14"/>
-      <c r="C14" t="s">
-        <v>23</v>
-      </c>
+      <c r="B14" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14"/>
       <c r="D14" s="2" t="n">
-        <v>32.6</v>
-      </c>
-      <c r="E14"/>
-      <c r="F14"/>
+        <v>36.2663366336634</v>
+      </c>
+      <c r="E14" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15"/>
       <c r="B15"/>
       <c r="C15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>40.2</v>
+        <v>32.6</v>
       </c>
       <c r="E15"/>
       <c r="F15"/>
@@ -715,10 +724,10 @@
       <c r="A16"/>
       <c r="B16"/>
       <c r="C16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>32.3</v>
+        <v>40.2</v>
       </c>
       <c r="E16"/>
       <c r="F16"/>
@@ -727,73 +736,69 @@
       <c r="A17"/>
       <c r="B17"/>
       <c r="C17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>21.9</v>
-      </c>
-      <c r="E17" t="s">
-        <v>26</v>
-      </c>
-      <c r="F17" t="s">
-        <v>19</v>
-      </c>
+        <v>32.3</v>
+      </c>
+      <c r="E17"/>
+      <c r="F17"/>
     </row>
     <row r="18">
       <c r="A18"/>
       <c r="B18"/>
       <c r="C18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>36.6</v>
-      </c>
-      <c r="E18"/>
-      <c r="F18"/>
+        <v>21.9</v>
+      </c>
+      <c r="E18" t="s">
+        <v>29</v>
+      </c>
+      <c r="F18" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19"/>
       <c r="B19"/>
       <c r="C19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>23.1</v>
-      </c>
-      <c r="E19" t="s">
-        <v>28</v>
-      </c>
-      <c r="F19" t="s">
-        <v>29</v>
-      </c>
+        <v>36.6</v>
+      </c>
+      <c r="E19"/>
+      <c r="F19"/>
     </row>
     <row r="20">
       <c r="A20"/>
       <c r="B20"/>
       <c r="C20" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>20.2</v>
-      </c>
-      <c r="E20"/>
-      <c r="F20"/>
+        <v>23.1</v>
+      </c>
+      <c r="E20" t="s">
+        <v>31</v>
+      </c>
+      <c r="F20" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21"/>
       <c r="B21"/>
       <c r="C21" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>25.2</v>
-      </c>
-      <c r="E21" t="s">
-        <v>32</v>
-      </c>
-      <c r="F21" t="s">
-        <v>33</v>
-      </c>
+        <v>20.2</v>
+      </c>
+      <c r="E21"/>
+      <c r="F21"/>
     </row>
     <row r="22">
       <c r="A22"/>
@@ -802,63 +807,67 @@
         <v>34</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>21.4</v>
-      </c>
-      <c r="E22"/>
-      <c r="F22"/>
+        <v>25.2</v>
+      </c>
+      <c r="E22" t="s">
+        <v>35</v>
+      </c>
+      <c r="F22" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23"/>
       <c r="B23"/>
       <c r="C23" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D23" s="2" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="E23"/>
+      <c r="F23"/>
+    </row>
+    <row r="24">
+      <c r="A24"/>
+      <c r="B24"/>
+      <c r="C24" t="s">
+        <v>38</v>
+      </c>
+      <c r="D24" s="2" t="n">
         <v>22.2</v>
       </c>
-      <c r="E23" t="s">
-        <v>36</v>
-      </c>
-      <c r="F23" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="s">
-        <v>37</v>
-      </c>
-      <c r="B24"/>
-      <c r="C24"/>
-      <c r="D24" s="2" t="n">
+      <c r="E24" t="s">
+        <v>39</v>
+      </c>
+      <c r="F24" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>40</v>
+      </c>
+      <c r="B25"/>
+      <c r="C25"/>
+      <c r="D25" s="2" t="n">
         <v>25.2727272727273</v>
       </c>
-      <c r="E24" t="s">
-        <v>38</v>
-      </c>
-      <c r="F24" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25"/>
-      <c r="B25"/>
-      <c r="C25" t="s">
-        <v>39</v>
-      </c>
-      <c r="D25" s="2" t="n">
-        <v>31.4</v>
-      </c>
-      <c r="E25"/>
-      <c r="F25"/>
+      <c r="E25" t="s">
+        <v>41</v>
+      </c>
+      <c r="F25" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26"/>
       <c r="B26"/>
       <c r="C26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>24.4</v>
+        <v>31.4</v>
       </c>
       <c r="E26"/>
       <c r="F26"/>
@@ -867,10 +876,10 @@
       <c r="A27"/>
       <c r="B27"/>
       <c r="C27" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>22.8</v>
+        <v>24.4</v>
       </c>
       <c r="E27"/>
       <c r="F27"/>
@@ -879,50 +888,50 @@
       <c r="A28"/>
       <c r="B28"/>
       <c r="C28" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>31</v>
+        <v>22.8</v>
       </c>
       <c r="E28"/>
       <c r="F28"/>
     </row>
     <row r="29">
-      <c r="A29" t="s">
-        <v>43</v>
-      </c>
+      <c r="A29"/>
       <c r="B29"/>
-      <c r="C29"/>
+      <c r="C29" t="s">
+        <v>45</v>
+      </c>
       <c r="D29" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="E29"/>
+      <c r="F29"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>46</v>
+      </c>
+      <c r="B30"/>
+      <c r="C30"/>
+      <c r="D30" s="2" t="n">
         <v>29.7507692307692</v>
       </c>
-      <c r="E29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F29" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30"/>
-      <c r="B30"/>
-      <c r="C30" t="s">
-        <v>45</v>
-      </c>
-      <c r="D30" s="2" t="n">
-        <v>29.8</v>
-      </c>
-      <c r="E30"/>
-      <c r="F30"/>
+      <c r="E30" t="s">
+        <v>6</v>
+      </c>
+      <c r="F30" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31"/>
       <c r="B31"/>
       <c r="C31" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>30.1</v>
+        <v>29.8</v>
       </c>
       <c r="E31"/>
       <c r="F31"/>
@@ -931,64 +940,80 @@
       <c r="A32"/>
       <c r="B32"/>
       <c r="C32" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>24.2</v>
+        <v>30.1</v>
       </c>
       <c r="E32"/>
       <c r="F32"/>
     </row>
     <row r="33">
-      <c r="A33" t="s">
-        <v>48</v>
-      </c>
+      <c r="A33"/>
       <c r="B33"/>
-      <c r="C33"/>
-      <c r="D33" s="2"/>
-      <c r="E33"/>
-      <c r="F33"/>
+      <c r="C33" t="s">
+        <v>7</v>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="E33" t="s">
+        <v>7</v>
+      </c>
+      <c r="F33" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="34">
-      <c r="A34"/>
+      <c r="A34" t="s">
+        <v>49</v>
+      </c>
       <c r="B34"/>
-      <c r="C34" t="s">
-        <v>49</v>
-      </c>
-      <c r="D34" s="2" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="E34" t="s">
-        <v>50</v>
-      </c>
-      <c r="F34" t="s">
-        <v>8</v>
-      </c>
+      <c r="C34"/>
+      <c r="D34" s="2"/>
+      <c r="E34"/>
+      <c r="F34"/>
     </row>
     <row r="35">
       <c r="A35"/>
       <c r="B35"/>
       <c r="C35" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>25.5</v>
+        <v>12.3</v>
       </c>
       <c r="E35" t="s">
         <v>51</v>
       </c>
       <c r="F35" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="37" ht="90" customHeight="1">
-      <c r="A37" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36"/>
+      <c r="B36"/>
+      <c r="C36" t="s">
         <v>52</v>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="E36" t="s">
+        <v>52</v>
+      </c>
+      <c r="F36" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="3" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A38:F38"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>